<commit_message>
Clean up age groups
</commit_message>
<xml_diff>
--- a/local/agegroups/USAW-Basic.xlsx
+++ b/local/agegroups/USAW-Basic.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10909"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/nemikor/usaw-owlcms/local/agegroups/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{726308BD-A237-DE46-86AC-6E61DA0A6EEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B063B2A-7AA5-1741-AACE-20A1683CA9EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="36840" yWindow="3160" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1540" yWindow="660" windowWidth="33020" windowHeight="21680" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="AgeGroups" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="78">
   <si>
     <t>code</t>
   </si>
@@ -177,12 +177,6 @@
     <t>Masters</t>
   </si>
   <si>
-    <t>Military</t>
-  </si>
-  <si>
-    <t>Military Masters</t>
-  </si>
-  <si>
     <t>#bodyweight categories for each age group (bodyweight category code followed by optional qualifying total, example: 45 80)</t>
   </si>
   <si>
@@ -277,30 +271,6 @@
   </si>
   <si>
     <t>QPoints</t>
-  </si>
-  <si>
-    <t>Adaptive - Hearing Youth</t>
-  </si>
-  <si>
-    <t>Adaptive - Hearing Masters</t>
-  </si>
-  <si>
-    <t>Adaptive - Vision Youth</t>
-  </si>
-  <si>
-    <t>Adaptive - Vision Masters</t>
-  </si>
-  <si>
-    <t>Adaptive - Physical Youth</t>
-  </si>
-  <si>
-    <t>Adaptive - Physical Masters</t>
-  </si>
-  <si>
-    <t>Adaptive - Intellectual Youth</t>
-  </si>
-  <si>
-    <t>Adaptive - Intellectual Masters</t>
   </si>
 </sst>
 </file>
@@ -670,7 +640,7 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>1</v>
@@ -685,7 +655,7 @@
         <v>4</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H1" s="3"/>
       <c r="I1" s="3"/>
@@ -2759,7 +2729,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{67E20EC9-CC14-8940-97C3-370B092B95BB}">
-  <dimension ref="A1:V15"/>
+  <dimension ref="A1:V5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="23.1640625" bestFit="1" customWidth="1"/>
@@ -2785,75 +2755,75 @@
   <sheetData>
     <row r="1" spans="1:22" x14ac:dyDescent="0.15">
       <c r="A1" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" t="s">
         <v>53</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
         <v>54</v>
       </c>
-      <c r="C1" t="s">
+      <c r="E1" t="s">
         <v>55</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>56</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>57</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>58</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>59</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>60</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>61</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>62</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>63</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>64</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>65</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>66</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>67</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>68</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>69</v>
       </c>
-      <c r="R1" t="s">
+      <c r="T1" t="s">
         <v>70</v>
       </c>
-      <c r="S1" t="s">
+      <c r="U1" t="s">
         <v>71</v>
       </c>
-      <c r="T1" t="s">
+      <c r="V1" t="s">
         <v>72</v>
-      </c>
-      <c r="U1" t="s">
-        <v>73</v>
-      </c>
-      <c r="V1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:22" ht="15" x14ac:dyDescent="0.2">
       <c r="A2" s="7" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B2" s="7" t="s">
         <v>6</v>
@@ -2865,10 +2835,10 @@
         <v>0</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="I2">
         <v>28</v>
@@ -2880,7 +2850,7 @@
         <v>23</v>
       </c>
       <c r="L2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M2">
         <v>999</v>
@@ -2907,7 +2877,7 @@
         <v>27</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C3" t="b">
         <v>0</v>
@@ -2916,10 +2886,10 @@
         <v>0</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F3" s="7" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="I3">
         <v>28</v>
@@ -2931,7 +2901,7 @@
         <v>23</v>
       </c>
       <c r="L3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M3">
         <v>999</v>
@@ -2967,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="I4">
         <v>28</v>
@@ -2982,7 +2952,7 @@
         <v>23</v>
       </c>
       <c r="L4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M4">
         <v>999</v>
@@ -3018,10 +2988,10 @@
         <v>0</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="F5" s="7" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="I5">
         <v>28</v>
@@ -3033,7 +3003,7 @@
         <v>23</v>
       </c>
       <c r="L5" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="M5">
         <v>999</v>
@@ -3052,510 +3022,6 @@
         <v>0</v>
       </c>
       <c r="S5">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="6" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A6" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="B6" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C6" t="b">
-        <v>0</v>
-      </c>
-      <c r="D6" t="b">
-        <v>0</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I6">
-        <v>28</v>
-      </c>
-      <c r="J6">
-        <v>25</v>
-      </c>
-      <c r="K6">
-        <v>23</v>
-      </c>
-      <c r="L6" t="s">
-        <v>77</v>
-      </c>
-      <c r="M6">
-        <v>999</v>
-      </c>
-      <c r="N6">
-        <v>2</v>
-      </c>
-      <c r="O6">
-        <v>5</v>
-      </c>
-      <c r="P6">
-        <v>5</v>
-      </c>
-      <c r="Q6" s="7"/>
-      <c r="R6" t="b">
-        <v>0</v>
-      </c>
-      <c r="S6">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A7" s="7" t="s">
-        <v>81</v>
-      </c>
-      <c r="B7" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C7" t="b">
-        <v>0</v>
-      </c>
-      <c r="D7" t="b">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F7" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7">
-        <v>28</v>
-      </c>
-      <c r="J7">
-        <v>25</v>
-      </c>
-      <c r="K7">
-        <v>23</v>
-      </c>
-      <c r="L7" t="s">
-        <v>77</v>
-      </c>
-      <c r="M7">
-        <v>999</v>
-      </c>
-      <c r="N7">
-        <v>2</v>
-      </c>
-      <c r="O7">
-        <v>5</v>
-      </c>
-      <c r="P7">
-        <v>5</v>
-      </c>
-      <c r="Q7" s="7"/>
-      <c r="R7" t="b">
-        <v>0</v>
-      </c>
-      <c r="S7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A8" s="7" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" t="b">
-        <v>0</v>
-      </c>
-      <c r="D8" t="b">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I8">
-        <v>28</v>
-      </c>
-      <c r="J8">
-        <v>25</v>
-      </c>
-      <c r="K8">
-        <v>23</v>
-      </c>
-      <c r="L8" t="s">
-        <v>77</v>
-      </c>
-      <c r="M8">
-        <v>999</v>
-      </c>
-      <c r="N8">
-        <v>2</v>
-      </c>
-      <c r="O8">
-        <v>5</v>
-      </c>
-      <c r="P8">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="7"/>
-      <c r="R8" t="b">
-        <v>0</v>
-      </c>
-      <c r="S8">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A9" s="7" t="s">
-        <v>87</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C9" t="b">
-        <v>0</v>
-      </c>
-      <c r="D9" t="b">
-        <v>0</v>
-      </c>
-      <c r="E9" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I9">
-        <v>28</v>
-      </c>
-      <c r="J9">
-        <v>25</v>
-      </c>
-      <c r="K9">
-        <v>23</v>
-      </c>
-      <c r="L9" t="s">
-        <v>77</v>
-      </c>
-      <c r="M9">
-        <v>999</v>
-      </c>
-      <c r="N9">
-        <v>2</v>
-      </c>
-      <c r="O9">
-        <v>5</v>
-      </c>
-      <c r="P9">
-        <v>5</v>
-      </c>
-      <c r="Q9" s="7"/>
-      <c r="R9" t="b">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="10" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A10" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C10" t="b">
-        <v>0</v>
-      </c>
-      <c r="D10" t="b">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I10">
-        <v>28</v>
-      </c>
-      <c r="J10">
-        <v>25</v>
-      </c>
-      <c r="K10">
-        <v>23</v>
-      </c>
-      <c r="L10" t="s">
-        <v>77</v>
-      </c>
-      <c r="M10">
-        <v>999</v>
-      </c>
-      <c r="N10">
-        <v>2</v>
-      </c>
-      <c r="O10">
-        <v>5</v>
-      </c>
-      <c r="P10">
-        <v>5</v>
-      </c>
-      <c r="Q10" s="7"/>
-      <c r="R10" t="b">
-        <v>0</v>
-      </c>
-      <c r="S10">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A11" s="7" t="s">
-        <v>85</v>
-      </c>
-      <c r="B11" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C11" t="b">
-        <v>0</v>
-      </c>
-      <c r="D11" t="b">
-        <v>0</v>
-      </c>
-      <c r="E11" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F11" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I11">
-        <v>28</v>
-      </c>
-      <c r="J11">
-        <v>25</v>
-      </c>
-      <c r="K11">
-        <v>23</v>
-      </c>
-      <c r="L11" t="s">
-        <v>77</v>
-      </c>
-      <c r="M11">
-        <v>999</v>
-      </c>
-      <c r="N11">
-        <v>2</v>
-      </c>
-      <c r="O11">
-        <v>5</v>
-      </c>
-      <c r="P11">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="7"/>
-      <c r="R11" t="b">
-        <v>0</v>
-      </c>
-      <c r="S11">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="12" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A12" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="B12" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" t="b">
-        <v>0</v>
-      </c>
-      <c r="D12" t="b">
-        <v>0</v>
-      </c>
-      <c r="E12" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="I12">
-        <v>28</v>
-      </c>
-      <c r="J12">
-        <v>25</v>
-      </c>
-      <c r="K12">
-        <v>23</v>
-      </c>
-      <c r="L12" t="s">
-        <v>77</v>
-      </c>
-      <c r="M12">
-        <v>999</v>
-      </c>
-      <c r="N12">
-        <v>2</v>
-      </c>
-      <c r="O12">
-        <v>5</v>
-      </c>
-      <c r="P12">
-        <v>5</v>
-      </c>
-      <c r="Q12" s="7"/>
-      <c r="R12" t="b">
-        <v>0</v>
-      </c>
-      <c r="S12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A13" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="B13" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C13" t="b">
-        <v>0</v>
-      </c>
-      <c r="D13" t="b">
-        <v>0</v>
-      </c>
-      <c r="E13" s="7" t="s">
-        <v>76</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I13">
-        <v>28</v>
-      </c>
-      <c r="J13">
-        <v>25</v>
-      </c>
-      <c r="K13">
-        <v>23</v>
-      </c>
-      <c r="L13" t="s">
-        <v>77</v>
-      </c>
-      <c r="M13">
-        <v>999</v>
-      </c>
-      <c r="N13">
-        <v>2</v>
-      </c>
-      <c r="O13">
-        <v>5</v>
-      </c>
-      <c r="P13">
-        <v>5</v>
-      </c>
-      <c r="Q13" s="7"/>
-      <c r="R13" t="b">
-        <v>0</v>
-      </c>
-      <c r="S13">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="14" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A14" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="B14" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" t="b">
-        <v>0</v>
-      </c>
-      <c r="D14" t="b">
-        <v>0</v>
-      </c>
-      <c r="E14" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>51</v>
-      </c>
-      <c r="I14">
-        <v>28</v>
-      </c>
-      <c r="J14">
-        <v>25</v>
-      </c>
-      <c r="K14">
-        <v>23</v>
-      </c>
-      <c r="M14">
-        <v>999</v>
-      </c>
-      <c r="N14">
-        <v>2</v>
-      </c>
-      <c r="O14">
-        <v>5</v>
-      </c>
-      <c r="P14">
-        <v>5</v>
-      </c>
-      <c r="Q14" s="7"/>
-      <c r="R14" t="b">
-        <v>0</v>
-      </c>
-      <c r="S14">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="15" spans="1:22" x14ac:dyDescent="0.15">
-      <c r="A15" s="7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B15" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="C15" t="b">
-        <v>0</v>
-      </c>
-      <c r="D15" t="b">
-        <v>0</v>
-      </c>
-      <c r="E15" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="I15">
-        <v>28</v>
-      </c>
-      <c r="J15">
-        <v>25</v>
-      </c>
-      <c r="K15">
-        <v>23</v>
-      </c>
-      <c r="M15">
-        <v>999</v>
-      </c>
-      <c r="N15">
-        <v>2</v>
-      </c>
-      <c r="O15">
-        <v>5</v>
-      </c>
-      <c r="P15">
-        <v>5</v>
-      </c>
-      <c r="Q15" s="7"/>
-      <c r="R15" t="b">
-        <v>0</v>
-      </c>
-      <c r="S15">
         <v>5</v>
       </c>
     </row>

</xml_diff>